<commit_message>
new column name TestName
</commit_message>
<xml_diff>
--- a/Dev_changeUnitsDxI9000.xlsx
+++ b/Dev_changeUnitsDxI9000.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="13125" windowHeight="6105"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="13130" windowHeight="6110"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet 1" sheetId="1" r:id="rId1"/>
@@ -24,9 +24,6 @@
     <t>TestOrderCode</t>
   </si>
   <si>
-    <t>DxI9000</t>
-  </si>
-  <si>
     <t>Einheit_9000</t>
   </si>
   <si>
@@ -205,13 +202,19 @@
   </si>
   <si>
     <t>PTHIO</t>
+  </si>
+  <si>
+    <t>TestName</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="2" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="165" formatCode="0.0"/>
+  </numFmts>
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -245,11 +248,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -547,750 +551,750 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:I37"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>1</v>
+        <v>61</v>
       </c>
       <c r="C1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
-        <v>3</v>
-      </c>
       <c r="E1" t="s">
+        <v>37</v>
+      </c>
+      <c r="F1" t="s">
         <v>38</v>
       </c>
-      <c r="F1" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:9">
       <c r="A2">
         <v>115</v>
       </c>
       <c r="B2" t="s">
+        <v>32</v>
+      </c>
+      <c r="C2" t="s">
         <v>33</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>34</v>
       </c>
-      <c r="D2" t="s">
-        <v>35</v>
-      </c>
       <c r="E2">
         <v>1</v>
       </c>
       <c r="F2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="I2" s="1"/>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9">
       <c r="A3">
         <v>116</v>
       </c>
       <c r="B3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C3" t="s">
+        <v>33</v>
+      </c>
+      <c r="D3" t="s">
         <v>34</v>
       </c>
-      <c r="D3" t="s">
-        <v>35</v>
-      </c>
       <c r="E3">
         <v>1</v>
       </c>
       <c r="F3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="I3" s="1"/>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9">
       <c r="A4">
         <v>119</v>
       </c>
       <c r="B4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" t="s">
         <v>8</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>9</v>
       </c>
-      <c r="D4" t="s">
-        <v>10</v>
-      </c>
       <c r="E4" t="s">
-        <v>40</v>
-      </c>
-      <c r="F4">
+        <v>39</v>
+      </c>
+      <c r="F4" s="2">
         <v>362.46</v>
       </c>
       <c r="I4" s="1"/>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9">
       <c r="A5">
         <v>128</v>
       </c>
       <c r="B5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C5" t="s">
+        <v>4</v>
+      </c>
+      <c r="D5" t="s">
         <v>5</v>
       </c>
-      <c r="D5" t="s">
-        <v>6</v>
-      </c>
       <c r="E5">
         <v>1</v>
       </c>
       <c r="F5" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="I5" s="1"/>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9">
       <c r="A6">
         <v>149</v>
       </c>
       <c r="B6" t="s">
+        <v>51</v>
+      </c>
+      <c r="C6" t="s">
         <v>52</v>
       </c>
-      <c r="C6" t="s">
-        <v>53</v>
-      </c>
       <c r="D6" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E6" t="s">
-        <v>40</v>
-      </c>
-      <c r="F6">
+        <v>39</v>
+      </c>
+      <c r="F6" s="2">
         <v>314.47000000000003</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9">
       <c r="A7">
         <v>156</v>
       </c>
       <c r="B7" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C7" t="s">
+        <v>4</v>
+      </c>
+      <c r="D7" t="s">
         <v>5</v>
       </c>
-      <c r="D7" t="s">
-        <v>6</v>
-      </c>
       <c r="E7">
         <v>1</v>
       </c>
       <c r="F7" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9">
       <c r="A8">
         <v>159</v>
       </c>
       <c r="B8" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C8" t="s">
+        <v>41</v>
+      </c>
+      <c r="D8" t="s">
         <v>42</v>
       </c>
-      <c r="D8" t="s">
-        <v>43</v>
-      </c>
       <c r="E8">
         <v>1</v>
       </c>
       <c r="F8" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9">
       <c r="A9">
         <v>162</v>
       </c>
       <c r="B9" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C9" t="s">
+        <v>4</v>
+      </c>
+      <c r="D9" t="s">
         <v>5</v>
       </c>
-      <c r="D9" t="s">
-        <v>6</v>
-      </c>
       <c r="E9">
         <v>1</v>
       </c>
       <c r="F9" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9">
       <c r="A10">
         <v>163</v>
       </c>
       <c r="B10" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C10" t="s">
+        <v>4</v>
+      </c>
+      <c r="D10" t="s">
         <v>5</v>
-      </c>
-      <c r="D10" t="s">
-        <v>6</v>
       </c>
       <c r="E10">
         <v>2</v>
       </c>
       <c r="F10" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9">
       <c r="A11">
         <v>175</v>
       </c>
       <c r="B11" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C11" t="s">
+        <v>41</v>
+      </c>
+      <c r="D11" t="s">
         <v>42</v>
       </c>
-      <c r="D11" t="s">
-        <v>43</v>
-      </c>
       <c r="E11">
         <v>1</v>
       </c>
       <c r="F11" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9">
       <c r="A12">
         <v>178</v>
       </c>
       <c r="B12" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C12" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D12" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E12">
         <v>1</v>
       </c>
       <c r="F12" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9">
       <c r="A13">
         <v>182</v>
       </c>
       <c r="B13" t="s">
+        <v>19</v>
+      </c>
+      <c r="C13" t="s">
         <v>20</v>
       </c>
-      <c r="C13" t="s">
+      <c r="D13" t="s">
         <v>21</v>
       </c>
-      <c r="D13" t="s">
-        <v>22</v>
-      </c>
       <c r="E13">
         <v>1</v>
       </c>
       <c r="F13" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9">
       <c r="A14">
         <v>190</v>
       </c>
       <c r="B14" t="s">
+        <v>29</v>
+      </c>
+      <c r="C14" t="s">
+        <v>15</v>
+      </c>
+      <c r="D14" t="s">
         <v>30</v>
       </c>
-      <c r="C14" t="s">
-        <v>16</v>
-      </c>
-      <c r="D14" t="s">
-        <v>31</v>
-      </c>
       <c r="E14">
         <v>1</v>
       </c>
       <c r="F14" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9">
       <c r="A15">
         <v>193</v>
       </c>
       <c r="B15" t="s">
+        <v>40</v>
+      </c>
+      <c r="C15" t="s">
         <v>41</v>
       </c>
-      <c r="C15" t="s">
+      <c r="D15" t="s">
         <v>42</v>
       </c>
-      <c r="D15" t="s">
-        <v>43</v>
-      </c>
       <c r="E15">
         <v>1</v>
       </c>
       <c r="F15" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9">
       <c r="A16">
         <v>195</v>
       </c>
       <c r="B16" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C16" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D16" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E16" t="s">
-        <v>40</v>
-      </c>
-      <c r="F16">
+        <v>39</v>
+      </c>
+      <c r="F16" s="2">
         <v>288.43099999999998</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6">
       <c r="A17">
         <v>209</v>
       </c>
       <c r="B17" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C17" t="s">
+        <v>33</v>
+      </c>
+      <c r="D17" t="s">
         <v>34</v>
       </c>
-      <c r="D17" t="s">
-        <v>35</v>
-      </c>
       <c r="E17">
         <v>1</v>
       </c>
       <c r="F17" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6">
       <c r="A18">
         <v>212</v>
       </c>
       <c r="B18" t="s">
+        <v>14</v>
+      </c>
+      <c r="C18" t="s">
         <v>15</v>
       </c>
-      <c r="C18" t="s">
+      <c r="D18" t="s">
         <v>16</v>
       </c>
-      <c r="D18" t="s">
-        <v>17</v>
-      </c>
       <c r="E18" t="s">
-        <v>40</v>
-      </c>
-      <c r="F18">
+        <v>39</v>
+      </c>
+      <c r="F18" s="2">
         <v>650.97699999999998</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6">
       <c r="A19">
         <v>214</v>
       </c>
       <c r="B19" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C19" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D19" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E19">
         <v>1</v>
       </c>
       <c r="F19" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6">
       <c r="A20">
         <v>215</v>
       </c>
       <c r="B20" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C20" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D20" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E20">
         <v>1</v>
       </c>
       <c r="F20" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6">
       <c r="A21">
         <v>226</v>
       </c>
       <c r="B21" t="s">
+        <v>17</v>
+      </c>
+      <c r="C21" t="s">
         <v>18</v>
       </c>
-      <c r="C21" t="s">
-        <v>19</v>
-      </c>
       <c r="D21" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E21" t="s">
-        <v>40</v>
-      </c>
-      <c r="F21">
+        <v>39</v>
+      </c>
+      <c r="F21" s="2">
         <v>776.87400000000002</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6">
       <c r="A22">
         <v>235</v>
       </c>
       <c r="B22" t="s">
+        <v>10</v>
+      </c>
+      <c r="C22" t="s">
+        <v>8</v>
+      </c>
+      <c r="D22" t="s">
         <v>11</v>
       </c>
-      <c r="C22" t="s">
-        <v>9</v>
-      </c>
-      <c r="D22" t="s">
-        <v>12</v>
-      </c>
       <c r="E22" t="s">
-        <v>40</v>
-      </c>
-      <c r="F22">
+        <v>39</v>
+      </c>
+      <c r="F22" s="2">
         <v>368.49</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:6">
       <c r="A23">
         <v>245</v>
       </c>
       <c r="B23" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C23" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D23" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E23">
         <v>1</v>
       </c>
       <c r="F23" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6">
       <c r="A24">
         <v>255</v>
       </c>
       <c r="B24" t="s">
+        <v>25</v>
+      </c>
+      <c r="C24" t="s">
         <v>26</v>
       </c>
-      <c r="C24" t="s">
-        <v>27</v>
-      </c>
       <c r="D24" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E24">
         <v>1</v>
       </c>
       <c r="F24" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6">
       <c r="A25">
         <v>292</v>
       </c>
       <c r="B25" t="s">
+        <v>49</v>
+      </c>
+      <c r="C25" t="s">
         <v>50</v>
       </c>
-      <c r="C25" t="s">
-        <v>51</v>
-      </c>
       <c r="D25" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E25" t="s">
-        <v>40</v>
-      </c>
-      <c r="F25">
+        <v>39</v>
+      </c>
+      <c r="F25" s="2">
         <v>272.39999999999998</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:6">
       <c r="A26">
         <v>293</v>
       </c>
       <c r="B26" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C26" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D26" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E26" t="s">
-        <v>40</v>
-      </c>
-      <c r="F26">
+        <v>39</v>
+      </c>
+      <c r="F26" s="2">
         <v>140000</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:6">
       <c r="A27">
         <v>299</v>
       </c>
       <c r="B27" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C27" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D27" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E27">
         <v>1</v>
       </c>
       <c r="F27" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6">
       <c r="A28">
         <v>1125</v>
       </c>
       <c r="B28" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C28" t="s">
+        <v>4</v>
+      </c>
+      <c r="D28" t="s">
         <v>5</v>
       </c>
-      <c r="D28" t="s">
-        <v>6</v>
-      </c>
       <c r="E28">
         <v>1</v>
       </c>
       <c r="F28" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6">
       <c r="A29">
         <v>1169</v>
       </c>
       <c r="B29" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C29" t="s">
+        <v>4</v>
+      </c>
+      <c r="D29" t="s">
         <v>5</v>
       </c>
-      <c r="D29" t="s">
-        <v>6</v>
-      </c>
       <c r="E29">
         <v>1</v>
       </c>
       <c r="F29" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6">
       <c r="A30">
         <v>1170</v>
       </c>
       <c r="B30" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C30" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D30" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E30">
         <v>1</v>
       </c>
       <c r="F30" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6">
       <c r="A31">
         <v>1180</v>
       </c>
       <c r="B31" t="s">
+        <v>3</v>
+      </c>
+      <c r="C31" t="s">
         <v>4</v>
       </c>
-      <c r="C31" t="s">
+      <c r="D31" t="s">
         <v>5</v>
       </c>
-      <c r="D31" t="s">
-        <v>6</v>
-      </c>
       <c r="E31">
         <v>1</v>
       </c>
       <c r="F31" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6">
       <c r="A32">
         <v>1200</v>
       </c>
       <c r="B32" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C32" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D32" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E32">
         <v>1</v>
       </c>
       <c r="F32" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6">
       <c r="A33">
         <v>1240</v>
       </c>
       <c r="B33" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C33" t="s">
+        <v>4</v>
+      </c>
+      <c r="D33" t="s">
         <v>5</v>
       </c>
-      <c r="D33" t="s">
-        <v>6</v>
-      </c>
       <c r="E33">
         <v>1</v>
       </c>
       <c r="F33" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6">
       <c r="A34">
         <v>1271</v>
       </c>
       <c r="B34" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C34" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D34" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E34" t="s">
-        <v>40</v>
-      </c>
-      <c r="F34">
+        <v>39</v>
+      </c>
+      <c r="F34" s="2">
         <v>400.64</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:6">
       <c r="A35">
         <v>1273</v>
       </c>
       <c r="B35" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C35" t="s">
+        <v>33</v>
+      </c>
+      <c r="D35" t="s">
         <v>34</v>
       </c>
-      <c r="D35" t="s">
-        <v>35</v>
-      </c>
       <c r="E35">
         <v>1</v>
       </c>
       <c r="F35" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6">
       <c r="A36">
         <v>1277</v>
       </c>
       <c r="B36" t="s">
+        <v>27</v>
+      </c>
+      <c r="C36" t="s">
+        <v>20</v>
+      </c>
+      <c r="D36" t="s">
         <v>28</v>
       </c>
-      <c r="C36" t="s">
-        <v>21</v>
-      </c>
-      <c r="D36" t="s">
-        <v>29</v>
-      </c>
       <c r="E36">
         <v>1</v>
       </c>
       <c r="F36" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6">
       <c r="A37">
         <v>1280</v>
       </c>
       <c r="B37" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C37" t="s">
+        <v>4</v>
+      </c>
+      <c r="D37" t="s">
         <v>5</v>
       </c>
-      <c r="D37" t="s">
-        <v>6</v>
-      </c>
       <c r="E37">
         <v>1</v>
       </c>
       <c r="F37" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
   </sheetData>

</xml_diff>